<commit_message>
Drop LilyGO T-Panel S3 support: Bosun runs on the Waveshare only
Removes the T-Panel display/touch driver (XL9535 init, CST3240), the
external buzzer options (PCF8574 backpack, GPIO) that only the T-Panel
needed, the t_panel_s3 build and CI target, and the board choice on the
installer page. board.h now holds only the Waveshare pins and refuses the
old board flags. The OTA page no longer mentions the T-Panel screen
(11 languages updated). README, LEESMIJ, COMPATIBILITEIT, quickstart and
the order list now describe the Waveshare only.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01DV9tygc5YXT9SuFFA2qLm4
</commit_message>
<xml_diff>
--- a/bestellijst.xlsx
+++ b/bestellijst.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bestellijst" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Bestellijst'!$A$4:$J$19</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Bestellijst'!$A$4:$J$18</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -468,7 +468,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J22"/>
+  <dimension ref="A1:J21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
@@ -552,7 +552,7 @@
     <row r="5">
       <c r="A5" s="5" t="inlineStr">
         <is>
-          <t>LILYGO T-Panel S3, CAN-versie (H720)</t>
+          <t>Waveshare ESP32-S3-Touch-LCD-4 (touchversie)</t>
         </is>
       </c>
       <c r="B5" s="5" t="n">
@@ -565,19 +565,19 @@
       </c>
       <c r="D5" s="5" t="inlineStr">
         <is>
-          <t>Het scherm met de ESP32-S3 en de CAN-aansluiting voor NMEA 2000</t>
+          <t>Het scherm met de ESP32-S3; CAN voor NMEA 2000, klok, zoemer en micro-SD zitten erop</t>
         </is>
       </c>
       <c r="E5" s="5" t="inlineStr">
         <is>
-          <t>T-Panel S3 H720 CAN FD</t>
+          <t>Waveshare ESP32-S3-Touch-LCD-4</t>
         </is>
       </c>
       <c r="F5" s="6" t="n">
+        <v>35</v>
+      </c>
+      <c r="G5" s="6" t="n">
         <v>55</v>
-      </c>
-      <c r="G5" s="6" t="n">
-        <v>90</v>
       </c>
       <c r="H5" s="6">
         <f>B5*F5</f>
@@ -589,14 +589,14 @@
       </c>
       <c r="J5" s="5" t="inlineStr">
         <is>
-          <t>Kies bewust H720 (CAN FD). De RS485-versie (H719) heeft geen CAN.</t>
+          <t>Neem de touchversie. Niet de -4B: die heeft geen CAN en geen 12 V-ingang.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
         <is>
-          <t>DS3231 RTC-module met CR2032-houder</t>
+          <t>Oplaadbare RTC-cel (ML1220) met stekkertje</t>
         </is>
       </c>
       <c r="B6" s="5" t="n">
@@ -609,19 +609,19 @@
       </c>
       <c r="D6" s="5" t="inlineStr">
         <is>
-          <t>Bewaart de tijd ook zonder stroom</t>
+          <t>Houdt de klok gaande zonder stroom</t>
         </is>
       </c>
       <c r="E6" s="5" t="inlineStr">
         <is>
-          <t>DS3231 RTC module CR2032</t>
+          <t>Waveshare RTC battery ML1220</t>
         </is>
       </c>
       <c r="F6" s="6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G6" s="6" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="H6" s="6">
         <f>B6*F6</f>
@@ -633,14 +633,14 @@
       </c>
       <c r="J6" s="5" t="inlineStr">
         <is>
-          <t>Controleer of de module een laadcircuit heeft (ZS-042). Zie de README over het diodetje/de weerstand.</t>
+          <t>Als optie bij Waveshare mee te bestellen. Geen gewone CR2032: het board laadt de cel bij.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="5" t="inlineStr">
         <is>
-          <t>CR2032 knoopcel</t>
+          <t>Zekering 1 A met houder</t>
         </is>
       </c>
       <c r="B7" s="5" t="n">
@@ -653,19 +653,19 @@
       </c>
       <c r="D7" s="5" t="inlineStr">
         <is>
-          <t>Voeding voor de klok</t>
+          <t>Beveiliging van de 12 V-voeding van het board</t>
         </is>
       </c>
       <c r="E7" s="5" t="inlineStr">
         <is>
-          <t>CR2032 3V lithium</t>
+          <t>inline fuse holder 1A blade</t>
         </is>
       </c>
       <c r="F7" s="6" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G7" s="6" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="H7" s="6">
         <f>B7*F7</f>
@@ -677,14 +677,14 @@
       </c>
       <c r="J7" s="5" t="inlineStr">
         <is>
-          <t>Neem een setje van 5. Ook voor later.</t>
+          <t>Plaats dicht bij de accu.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="5" t="inlineStr">
         <is>
-          <t>I2C LCD-backpack PCF8574 (voor 1602/2004)</t>
+          <t>Draad 1 mm² en 2,5 mm², met krimpkousen en kabelschoenen</t>
         </is>
       </c>
       <c r="B8" s="5" t="n">
@@ -697,19 +697,19 @@
       </c>
       <c r="D8" s="5" t="inlineStr">
         <is>
-          <t>Biedt de I2C-poort en de pinnen voor de zoemer. Het LCD-scherm zelf hoef je niet te kopen.</t>
+          <t>Voeding en signaalbedrading</t>
         </is>
       </c>
       <c r="E8" s="5" t="inlineStr">
         <is>
-          <t>PCF8574 I2C LCD backpack 1602</t>
+          <t>kabelschoen krimpset</t>
         </is>
       </c>
       <c r="F8" s="6" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="G8" s="6" t="n">
-        <v>4</v>
+        <v>12</v>
       </c>
       <c r="H8" s="6">
         <f>B8*F8</f>
@@ -721,14 +721,14 @@
       </c>
       <c r="J8" s="5" t="inlineStr">
         <is>
-          <t>Met de 16-polige header; de pinnen 15 en 16 zijn nodig voor de zoemer.</t>
+          <t>De stroomdraad naar de klem 2,5 mm² of dikker.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="5" t="inlineStr">
         <is>
-          <t>Actieve zoemer 3-5 V</t>
+          <t>NMEA 2000 drop-kabel met M12-stekker</t>
         </is>
       </c>
       <c r="B9" s="5" t="n">
@@ -741,19 +741,19 @@
       </c>
       <c r="D9" s="5" t="inlineStr">
         <is>
-          <t>Piept bij een rood alarm</t>
+          <t>Verbindt het board met de bus van je boot</t>
         </is>
       </c>
       <c r="E9" s="5" t="inlineStr">
         <is>
-          <t>active buzzer 5V</t>
+          <t>NMEA 2000 drop cable M12 female</t>
         </is>
       </c>
       <c r="F9" s="6" t="n">
-        <v>1</v>
+        <v>15</v>
       </c>
       <c r="G9" s="6" t="n">
-        <v>3</v>
+        <v>30</v>
       </c>
       <c r="H9" s="6">
         <f>B9*F9</f>
@@ -765,14 +765,14 @@
       </c>
       <c r="J9" s="5" t="inlineStr">
         <is>
-          <t>Actief, dus met een eigen oscillator. Een passieve zoemer piept niet vanzelf.</t>
+          <t>Een kabel met één open einde. Lengte: tot aan de bus.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
         <is>
-          <t>Zekering 1 A met houder</t>
+          <t>NMEA 2000 T-stuk of afsluiter</t>
         </is>
       </c>
       <c r="B10" s="5" t="n">
@@ -780,24 +780,24 @@
       </c>
       <c r="C10" s="5" t="inlineStr">
         <is>
-          <t>Ja</t>
+          <t>Soms nodig</t>
         </is>
       </c>
       <c r="D10" s="5" t="inlineStr">
         <is>
-          <t>Beveiliging van de 12 V-voeding van het board</t>
+          <t>Zodat je kabel op de bus kan zitten</t>
         </is>
       </c>
       <c r="E10" s="5" t="inlineStr">
         <is>
-          <t>inline fuse holder 1A blade</t>
+          <t>NMEA 2000 T-piece</t>
         </is>
       </c>
       <c r="F10" s="6" t="n">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="G10" s="6" t="n">
-        <v>6</v>
+        <v>20</v>
       </c>
       <c r="H10" s="6">
         <f>B10*F10</f>
@@ -809,14 +809,14 @@
       </c>
       <c r="J10" s="5" t="inlineStr">
         <is>
-          <t>Plaats dicht bij de accu.</t>
+          <t>Let op: er mag maar één afsluiter per uiteinde van de bus zitten.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="5" t="inlineStr">
         <is>
-          <t>Draad 1 mm² en 2,5 mm², met krimpkousen en kabelschoenen</t>
+          <t>USB-C datakabel</t>
         </is>
       </c>
       <c r="B11" s="5" t="n">
@@ -829,19 +829,19 @@
       </c>
       <c r="D11" s="5" t="inlineStr">
         <is>
-          <t>Voeding en signaalbedrading</t>
+          <t>Firmware zetten en de seriële log bekijken</t>
         </is>
       </c>
       <c r="E11" s="5" t="inlineStr">
         <is>
-          <t>kabelschoen krimpset</t>
+          <t>USB-C datakabel</t>
         </is>
       </c>
       <c r="F11" s="6" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="G11" s="6" t="n">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="H11" s="6">
         <f>B11*F11</f>
@@ -853,14 +853,14 @@
       </c>
       <c r="J11" s="5" t="inlineStr">
         <is>
-          <t>De stroomdraad naar de klem 2,5 mm² of dikker.</t>
+          <t>Een kabel die data kan, geen alleen-laadkabel.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
         <is>
-          <t>NMEA 2000 drop-kabel met M12-stekker</t>
+          <t>Multimeter</t>
         </is>
       </c>
       <c r="B12" s="5" t="n">
@@ -868,24 +868,24 @@
       </c>
       <c r="C12" s="5" t="inlineStr">
         <is>
-          <t>Ja (CAN-versie)</t>
+          <t>Ja</t>
         </is>
       </c>
       <c r="D12" s="5" t="inlineStr">
         <is>
-          <t>Verbindt de T-Panel met de bus van je boot</t>
+          <t>Controleren van spanning, de bus en de afsluitweerstand (60 Ω)</t>
         </is>
       </c>
       <c r="E12" s="5" t="inlineStr">
         <is>
-          <t>NMEA 2000 drop cable M12 female</t>
+          <t>multimeter</t>
         </is>
       </c>
       <c r="F12" s="6" t="n">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="G12" s="6" t="n">
-        <v>30</v>
+        <v>25</v>
       </c>
       <c r="H12" s="6">
         <f>B12*F12</f>
@@ -897,14 +897,14 @@
       </c>
       <c r="J12" s="5" t="inlineStr">
         <is>
-          <t>Een kabel met één open einde. Lengte: tot aan de bus.</t>
+          <t>Een gewone multimeter is genoeg.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="5" t="inlineStr">
         <is>
-          <t>NMEA 2000 T-stuk of afsluiter</t>
+          <t>Micro-SD-kaart (FAT32, tot 32 GB)</t>
         </is>
       </c>
       <c r="B13" s="5" t="n">
@@ -912,24 +912,24 @@
       </c>
       <c r="C13" s="5" t="inlineStr">
         <is>
-          <t>Soms nodig</t>
+          <t>Optioneel</t>
         </is>
       </c>
       <c r="D13" s="5" t="inlineStr">
         <is>
-          <t>Zodat je kabel op de bus kan zitten</t>
+          <t>Metingen, logboek en backups</t>
         </is>
       </c>
       <c r="E13" s="5" t="inlineStr">
         <is>
-          <t>NMEA 2000 T-piece</t>
+          <t>micro SD 16GB</t>
         </is>
       </c>
       <c r="F13" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="G13" s="6" t="n">
         <v>10</v>
-      </c>
-      <c r="G13" s="6" t="n">
-        <v>20</v>
       </c>
       <c r="H13" s="6">
         <f>B13*F13</f>
@@ -941,36 +941,36 @@
       </c>
       <c r="J13" s="5" t="inlineStr">
         <is>
-          <t>Let op: er mag maar één afsluiter per uiteinde van de bus zitten.</t>
+          <t>Een kaart van 8 tot 32 GB is ruim genoeg.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="5" t="inlineStr">
         <is>
-          <t>USB-C datakabel</t>
+          <t>BME280-module (luchtdruk)</t>
         </is>
       </c>
       <c r="B14" s="5" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C14" s="5" t="inlineStr">
         <is>
-          <t>Ja</t>
+          <t>Optioneel</t>
         </is>
       </c>
       <c r="D14" s="5" t="inlineStr">
         <is>
-          <t>Firmware zetten en de seriële log bekijken</t>
+          <t>Barometer en stormwaarschuwing</t>
         </is>
       </c>
       <c r="E14" s="5" t="inlineStr">
         <is>
-          <t>USB-C datakabel</t>
+          <t>BME280 I2C module</t>
         </is>
       </c>
       <c r="F14" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G14" s="6" t="n">
         <v>8</v>
@@ -985,39 +985,39 @@
       </c>
       <c r="J14" s="5" t="inlineStr">
         <is>
-          <t>Een kabel die data kan, geen alleen-laadkabel.</t>
+          <t>Aantal 0: zelf optellen. Op de I2C-klem van het board.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="5" t="inlineStr">
         <is>
-          <t>Multimeter</t>
+          <t>Ruuvi-tag (temperatuur/vocht)</t>
         </is>
       </c>
       <c r="B15" s="5" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C15" s="5" t="inlineStr">
         <is>
-          <t>Ja</t>
+          <t>Optioneel</t>
         </is>
       </c>
       <c r="D15" s="5" t="inlineStr">
         <is>
-          <t>Controleren van spanning, de bus en de afsluitweerstand (60 Ω)</t>
+          <t>Draadloze thermometer, bv. voor de koelkast</t>
         </is>
       </c>
       <c r="E15" s="5" t="inlineStr">
         <is>
-          <t>multimeter</t>
+          <t>RuuviTag</t>
         </is>
       </c>
       <c r="F15" s="6" t="n">
-        <v>10</v>
+        <v>25</v>
       </c>
       <c r="G15" s="6" t="n">
-        <v>25</v>
+        <v>35</v>
       </c>
       <c r="H15" s="6">
         <f>B15*F15</f>
@@ -1029,14 +1029,14 @@
       </c>
       <c r="J15" s="5" t="inlineStr">
         <is>
-          <t>Een gewone multimeter is genoeg.</t>
+          <t>Aantal 0: per stuk zelf optellen. Geen bedrading, geen sleutel.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="5" t="inlineStr">
         <is>
-          <t>Ruuvi-tag (temperatuur/vocht)</t>
+          <t>Xiaomi LYWSD03MMC thermometer</t>
         </is>
       </c>
       <c r="B16" s="5" t="n">
@@ -1049,19 +1049,19 @@
       </c>
       <c r="D16" s="5" t="inlineStr">
         <is>
-          <t>Draadloze thermometer, bv. voor de koelkast</t>
+          <t>Goedkope draadloze thermometer</t>
         </is>
       </c>
       <c r="E16" s="5" t="inlineStr">
         <is>
-          <t>RuuviTag</t>
+          <t>LYWSD03MMC</t>
         </is>
       </c>
       <c r="F16" s="6" t="n">
-        <v>25</v>
+        <v>8</v>
       </c>
       <c r="G16" s="6" t="n">
-        <v>35</v>
+        <v>12</v>
       </c>
       <c r="H16" s="6">
         <f>B16*F16</f>
@@ -1073,14 +1073,14 @@
       </c>
       <c r="J16" s="5" t="inlineStr">
         <is>
-          <t>Aantal 0: per stuk zelf optellen. Geen bedrading, geen sleutel.</t>
+          <t>Aantal 0: per stuk zelf optellen. Eerst de ATC-firmware flashen; zie de README.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="5" t="inlineStr">
         <is>
-          <t>Xiaomi LYWSD03MMC thermometer</t>
+          <t>Mopeka Pro Check tanksensor</t>
         </is>
       </c>
       <c r="B17" s="5" t="n">
@@ -1093,19 +1093,19 @@
       </c>
       <c r="D17" s="5" t="inlineStr">
         <is>
-          <t>Goedkope draadloze thermometer</t>
+          <t>Tankniveau via de tankwand, bv. gas, water of diesel</t>
         </is>
       </c>
       <c r="E17" s="5" t="inlineStr">
         <is>
-          <t>LYWSD03MMC</t>
+          <t>Mopeka Pro Check</t>
         </is>
       </c>
       <c r="F17" s="6" t="n">
-        <v>8</v>
+        <v>45</v>
       </c>
       <c r="G17" s="6" t="n">
-        <v>12</v>
+        <v>70</v>
       </c>
       <c r="H17" s="6">
         <f>B17*F17</f>
@@ -1117,39 +1117,39 @@
       </c>
       <c r="J17" s="5" t="inlineStr">
         <is>
-          <t>Aantal 0: per stuk zelf optellen. Eerst de ATC-firmware flashen; zie de README.</t>
+          <t>Aantal 0: per tank zelf optellen. Kalibreren op vol en leeg.</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="5" t="inlineStr">
         <is>
-          <t>Mopeka Pro Check tanksensor</t>
+          <t>Behuizing (3D-print)</t>
         </is>
       </c>
       <c r="B18" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>Optioneel</t>
+        </is>
+      </c>
+      <c r="D18" s="5" t="inlineStr">
+        <is>
+          <t>Opbouw tegen een wand of inbouw in een schot</t>
+        </is>
+      </c>
+      <c r="E18" s="5" t="inlineStr">
+        <is>
+          <t>PETG of ASA filament</t>
+        </is>
+      </c>
+      <c r="F18" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="C18" s="5" t="inlineStr">
-        <is>
-          <t>Optioneel</t>
-        </is>
-      </c>
-      <c r="D18" s="5" t="inlineStr">
-        <is>
-          <t>Tankniveau via de tankwand, bv. gas (propaan)</t>
-        </is>
-      </c>
-      <c r="E18" s="5" t="inlineStr">
-        <is>
-          <t>Mopeka Pro Check</t>
-        </is>
-      </c>
-      <c r="F18" s="6" t="n">
-        <v>45</v>
-      </c>
       <c r="G18" s="6" t="n">
-        <v>70</v>
+        <v>5</v>
       </c>
       <c r="H18" s="6">
         <f>B18*F18</f>
@@ -1161,86 +1161,42 @@
       </c>
       <c r="J18" s="5" t="inlineStr">
         <is>
-          <t>Aantal 0: per tank zelf optellen. Kalibreren op vol en leeg.</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="5" t="inlineStr">
-        <is>
-          <t>Montagebeugel of kast voor het scherm</t>
-        </is>
-      </c>
-      <c r="B19" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="C19" s="5" t="inlineStr">
-        <is>
-          <t>Optioneel</t>
-        </is>
-      </c>
-      <c r="D19" s="5" t="inlineStr">
-        <is>
-          <t>Het board vastzetten</t>
-        </is>
-      </c>
-      <c r="E19" s="5" t="inlineStr">
-        <is>
-          <t>T-Panel mounting bracket</t>
-        </is>
-      </c>
-      <c r="F19" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="G19" s="6" t="n">
-        <v>25</v>
-      </c>
-      <c r="H19" s="6">
-        <f>B19*F19</f>
-        <v/>
-      </c>
-      <c r="I19" s="6">
-        <f>B19*G19</f>
-        <v/>
-      </c>
-      <c r="J19" s="5" t="inlineStr">
-        <is>
-          <t>Het project bevat ook behuizingsbestanden in de map structure.</t>
-        </is>
+          <t>Ontwerp in de map enclosure van het project; print in PETG of ASA (PLA wordt te zacht in de zon).</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="7" t="inlineStr">
+        <is>
+          <t>Totaal verplicht</t>
+        </is>
+      </c>
+      <c r="H20" s="8">
+        <f>SUMIF(C5:C18,"Ja*",H5:H18)</f>
+        <v/>
+      </c>
+      <c r="I20" s="8">
+        <f>SUMIF(C5:C18,"Ja*",I5:I18)</f>
+        <v/>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="7" t="inlineStr">
-        <is>
-          <t>Totaal verplicht</t>
-        </is>
-      </c>
-      <c r="H21" s="8">
-        <f>SUMIF(C5:C19,"Ja*",H5:H19)</f>
-        <v/>
-      </c>
-      <c r="I21" s="8">
-        <f>SUMIF(C5:C19,"Ja*",I5:I19)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
+      <c r="A21" t="inlineStr">
         <is>
           <t>Totaal soms nodig en optioneel (sensoren tellen per stuk, zie opmerking)</t>
         </is>
       </c>
-      <c r="H22" s="9">
-        <f>SUM(H5:H19)-H21</f>
-        <v/>
-      </c>
-      <c r="I22" s="9">
-        <f>SUM(I5:I19)-I21</f>
+      <c r="H21" s="9">
+        <f>SUM(H5:H18)-H20</f>
+        <v/>
+      </c>
+      <c r="I21" s="9">
+        <f>SUM(I5:I18)-I20</f>
         <v/>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A4:J19"/>
+  <autoFilter ref="A4:J18"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Docs: DFRobot SEN0236 as barometer sensor, wire ferrules everywhere
Recommend the DFRobot Gravity BME280 (SEN0236): locking connector on the
sensor side and no soldering, unlike loose GY-BME280 modules whose push-on
pins shake loose on a boat. README, LEESMIJ, both compatibility lists and
the order list mention it, plus a ferrule set with crimp tool for every
wire in the screw terminal.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01DV9tygc5YXT9SuFFA2qLm4
</commit_message>
<xml_diff>
--- a/bestellijst.xlsx
+++ b/bestellijst.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bestellijst" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Bestellijst'!$A$4:$J$18</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Bestellijst'!$A$4:$J$19</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -468,7 +468,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J21"/>
+  <dimension ref="A1:J22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
@@ -728,7 +728,7 @@
     <row r="9">
       <c r="A9" s="5" t="inlineStr">
         <is>
-          <t>NMEA 2000 drop-kabel met M12-stekker</t>
+          <t>Adereindhulzen 0,25–1,5 mm² met krimptang (set)</t>
         </is>
       </c>
       <c r="B9" s="5" t="n">
@@ -741,16 +741,16 @@
       </c>
       <c r="D9" s="5" t="inlineStr">
         <is>
-          <t>Verbindt het board met de bus van je boot</t>
+          <t>Op elke draad in de schroefklem: blijft vast bij trillingen</t>
         </is>
       </c>
       <c r="E9" s="5" t="inlineStr">
         <is>
-          <t>NMEA 2000 drop cable M12 female</t>
+          <t>adereindhulzen set krimptang</t>
         </is>
       </c>
       <c r="F9" s="6" t="n">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="G9" s="6" t="n">
         <v>30</v>
@@ -765,14 +765,14 @@
       </c>
       <c r="J9" s="5" t="inlineStr">
         <is>
-          <t>Een kabel met één open einde. Lengte: tot aan de bus.</t>
+          <t>Ook 0,25 mm² voor de dunne sensorkabel en een paar dubbele (twin) hulzen 2 × 0,5 mm².</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
         <is>
-          <t>NMEA 2000 T-stuk of afsluiter</t>
+          <t>NMEA 2000 drop-kabel met M12-stekker</t>
         </is>
       </c>
       <c r="B10" s="5" t="n">
@@ -780,24 +780,24 @@
       </c>
       <c r="C10" s="5" t="inlineStr">
         <is>
-          <t>Soms nodig</t>
+          <t>Ja</t>
         </is>
       </c>
       <c r="D10" s="5" t="inlineStr">
         <is>
-          <t>Zodat je kabel op de bus kan zitten</t>
+          <t>Verbindt het board met de bus van je boot</t>
         </is>
       </c>
       <c r="E10" s="5" t="inlineStr">
         <is>
-          <t>NMEA 2000 T-piece</t>
+          <t>NMEA 2000 drop cable M12 female</t>
         </is>
       </c>
       <c r="F10" s="6" t="n">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="G10" s="6" t="n">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="H10" s="6">
         <f>B10*F10</f>
@@ -809,14 +809,14 @@
       </c>
       <c r="J10" s="5" t="inlineStr">
         <is>
-          <t>Let op: er mag maar één afsluiter per uiteinde van de bus zitten.</t>
+          <t>Een kabel met één open einde. Lengte: tot aan de bus.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="5" t="inlineStr">
         <is>
-          <t>USB-C datakabel</t>
+          <t>NMEA 2000 T-stuk of afsluiter</t>
         </is>
       </c>
       <c r="B11" s="5" t="n">
@@ -824,24 +824,24 @@
       </c>
       <c r="C11" s="5" t="inlineStr">
         <is>
-          <t>Ja</t>
+          <t>Soms nodig</t>
         </is>
       </c>
       <c r="D11" s="5" t="inlineStr">
         <is>
-          <t>Firmware zetten en de seriële log bekijken</t>
+          <t>Zodat je kabel op de bus kan zitten</t>
         </is>
       </c>
       <c r="E11" s="5" t="inlineStr">
         <is>
-          <t>USB-C datakabel</t>
+          <t>NMEA 2000 T-piece</t>
         </is>
       </c>
       <c r="F11" s="6" t="n">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="G11" s="6" t="n">
-        <v>8</v>
+        <v>20</v>
       </c>
       <c r="H11" s="6">
         <f>B11*F11</f>
@@ -853,14 +853,14 @@
       </c>
       <c r="J11" s="5" t="inlineStr">
         <is>
-          <t>Een kabel die data kan, geen alleen-laadkabel.</t>
+          <t>Let op: er mag maar één afsluiter per uiteinde van de bus zitten.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
         <is>
-          <t>Multimeter</t>
+          <t>USB-C datakabel</t>
         </is>
       </c>
       <c r="B12" s="5" t="n">
@@ -873,19 +873,19 @@
       </c>
       <c r="D12" s="5" t="inlineStr">
         <is>
-          <t>Controleren van spanning, de bus en de afsluitweerstand (60 Ω)</t>
+          <t>Firmware zetten en de seriële log bekijken</t>
         </is>
       </c>
       <c r="E12" s="5" t="inlineStr">
         <is>
-          <t>multimeter</t>
+          <t>USB-C datakabel</t>
         </is>
       </c>
       <c r="F12" s="6" t="n">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="G12" s="6" t="n">
-        <v>25</v>
+        <v>8</v>
       </c>
       <c r="H12" s="6">
         <f>B12*F12</f>
@@ -897,14 +897,14 @@
       </c>
       <c r="J12" s="5" t="inlineStr">
         <is>
-          <t>Een gewone multimeter is genoeg.</t>
+          <t>Een kabel die data kan, geen alleen-laadkabel.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="5" t="inlineStr">
         <is>
-          <t>Micro-SD-kaart (FAT32, tot 32 GB)</t>
+          <t>Multimeter</t>
         </is>
       </c>
       <c r="B13" s="5" t="n">
@@ -912,24 +912,24 @@
       </c>
       <c r="C13" s="5" t="inlineStr">
         <is>
-          <t>Optioneel</t>
+          <t>Ja</t>
         </is>
       </c>
       <c r="D13" s="5" t="inlineStr">
         <is>
-          <t>Metingen, logboek en backups</t>
+          <t>Controleren van spanning, de bus en de afsluitweerstand (60 Ω)</t>
         </is>
       </c>
       <c r="E13" s="5" t="inlineStr">
         <is>
-          <t>micro SD 16GB</t>
+          <t>multimeter</t>
         </is>
       </c>
       <c r="F13" s="6" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="G13" s="6" t="n">
-        <v>10</v>
+        <v>25</v>
       </c>
       <c r="H13" s="6">
         <f>B13*F13</f>
@@ -941,18 +941,18 @@
       </c>
       <c r="J13" s="5" t="inlineStr">
         <is>
-          <t>Een kaart van 8 tot 32 GB is ruim genoeg.</t>
+          <t>Een gewone multimeter is genoeg.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="5" t="inlineStr">
         <is>
-          <t>BME280-module (luchtdruk)</t>
+          <t>Micro-SD-kaart (FAT32, tot 32 GB)</t>
         </is>
       </c>
       <c r="B14" s="5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C14" s="5" t="inlineStr">
         <is>
@@ -961,19 +961,19 @@
       </c>
       <c r="D14" s="5" t="inlineStr">
         <is>
-          <t>Barometer en stormwaarschuwing</t>
+          <t>Metingen, logboek en backups</t>
         </is>
       </c>
       <c r="E14" s="5" t="inlineStr">
         <is>
-          <t>BME280 I2C module</t>
+          <t>micro SD 16GB</t>
         </is>
       </c>
       <c r="F14" s="6" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="G14" s="6" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="H14" s="6">
         <f>B14*F14</f>
@@ -985,14 +985,14 @@
       </c>
       <c r="J14" s="5" t="inlineStr">
         <is>
-          <t>Aantal 0: zelf optellen. Op de I2C-klem van het board.</t>
+          <t>Een kaart van 8 tot 32 GB is ruim genoeg.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="5" t="inlineStr">
         <is>
-          <t>Ruuvi-tag (temperatuur/vocht)</t>
+          <t>DFRobot Gravity BME280 (SEN0236)</t>
         </is>
       </c>
       <c r="B15" s="5" t="n">
@@ -1005,19 +1005,19 @@
       </c>
       <c r="D15" s="5" t="inlineStr">
         <is>
-          <t>Draadloze thermometer, bv. voor de koelkast</t>
+          <t>Barometer en stormwaarschuwing (luchtdruk, ook vocht en temperatuur)</t>
         </is>
       </c>
       <c r="E15" s="5" t="inlineStr">
         <is>
-          <t>RuuviTag</t>
+          <t>DFRobot SEN0236</t>
         </is>
       </c>
       <c r="F15" s="6" t="n">
-        <v>25</v>
+        <v>15</v>
       </c>
       <c r="G15" s="6" t="n">
-        <v>35</v>
+        <v>20</v>
       </c>
       <c r="H15" s="6">
         <f>B15*F15</f>
@@ -1029,14 +1029,14 @@
       </c>
       <c r="J15" s="5" t="inlineStr">
         <is>
-          <t>Aantal 0: per stuk zelf optellen. Geen bedrading, geen sleutel.</t>
+          <t>Aantal 0: zelf optellen. Vergrendelende stekker, niets solderen. Dupont-stekkertje van de kabel afknippen, adereindhulzen erop, in de I2C-klem.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="5" t="inlineStr">
         <is>
-          <t>Xiaomi LYWSD03MMC thermometer</t>
+          <t>Ruuvi-tag (temperatuur/vocht)</t>
         </is>
       </c>
       <c r="B16" s="5" t="n">
@@ -1049,19 +1049,19 @@
       </c>
       <c r="D16" s="5" t="inlineStr">
         <is>
-          <t>Goedkope draadloze thermometer</t>
+          <t>Draadloze thermometer, bv. voor de koelkast</t>
         </is>
       </c>
       <c r="E16" s="5" t="inlineStr">
         <is>
-          <t>LYWSD03MMC</t>
+          <t>RuuviTag</t>
         </is>
       </c>
       <c r="F16" s="6" t="n">
-        <v>8</v>
+        <v>25</v>
       </c>
       <c r="G16" s="6" t="n">
-        <v>12</v>
+        <v>35</v>
       </c>
       <c r="H16" s="6">
         <f>B16*F16</f>
@@ -1073,14 +1073,14 @@
       </c>
       <c r="J16" s="5" t="inlineStr">
         <is>
-          <t>Aantal 0: per stuk zelf optellen. Eerst de ATC-firmware flashen; zie de README.</t>
+          <t>Aantal 0: per stuk zelf optellen. Geen bedrading, geen sleutel.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="5" t="inlineStr">
         <is>
-          <t>Mopeka Pro Check tanksensor</t>
+          <t>Xiaomi LYWSD03MMC thermometer</t>
         </is>
       </c>
       <c r="B17" s="5" t="n">
@@ -1093,19 +1093,19 @@
       </c>
       <c r="D17" s="5" t="inlineStr">
         <is>
-          <t>Tankniveau via de tankwand, bv. gas, water of diesel</t>
+          <t>Goedkope draadloze thermometer</t>
         </is>
       </c>
       <c r="E17" s="5" t="inlineStr">
         <is>
-          <t>Mopeka Pro Check</t>
+          <t>LYWSD03MMC</t>
         </is>
       </c>
       <c r="F17" s="6" t="n">
-        <v>45</v>
+        <v>8</v>
       </c>
       <c r="G17" s="6" t="n">
-        <v>70</v>
+        <v>12</v>
       </c>
       <c r="H17" s="6">
         <f>B17*F17</f>
@@ -1117,18 +1117,18 @@
       </c>
       <c r="J17" s="5" t="inlineStr">
         <is>
-          <t>Aantal 0: per tank zelf optellen. Kalibreren op vol en leeg.</t>
+          <t>Aantal 0: per stuk zelf optellen. Eerst de ATC-firmware flashen; zie de README.</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="5" t="inlineStr">
         <is>
-          <t>Behuizing (3D-print)</t>
+          <t>Mopeka Pro Check tanksensor</t>
         </is>
       </c>
       <c r="B18" s="5" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C18" s="5" t="inlineStr">
         <is>
@@ -1137,19 +1137,19 @@
       </c>
       <c r="D18" s="5" t="inlineStr">
         <is>
-          <t>Opbouw tegen een wand of inbouw in een schot</t>
+          <t>Tankniveau via de tankwand, bv. gas, water of diesel</t>
         </is>
       </c>
       <c r="E18" s="5" t="inlineStr">
         <is>
-          <t>PETG of ASA filament</t>
+          <t>Mopeka Pro Check</t>
         </is>
       </c>
       <c r="F18" s="6" t="n">
-        <v>0</v>
+        <v>45</v>
       </c>
       <c r="G18" s="6" t="n">
-        <v>5</v>
+        <v>70</v>
       </c>
       <c r="H18" s="6">
         <f>B18*F18</f>
@@ -1161,42 +1161,86 @@
       </c>
       <c r="J18" s="5" t="inlineStr">
         <is>
+          <t>Aantal 0: per tank zelf optellen. Kalibreren op vol en leeg.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="5" t="inlineStr">
+        <is>
+          <t>Behuizing (3D-print)</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="C19" s="5" t="inlineStr">
+        <is>
+          <t>Optioneel</t>
+        </is>
+      </c>
+      <c r="D19" s="5" t="inlineStr">
+        <is>
+          <t>Opbouw tegen een wand of inbouw in een schot</t>
+        </is>
+      </c>
+      <c r="E19" s="5" t="inlineStr">
+        <is>
+          <t>PETG of ASA filament</t>
+        </is>
+      </c>
+      <c r="F19" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="G19" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="H19" s="6">
+        <f>B19*F19</f>
+        <v/>
+      </c>
+      <c r="I19" s="6">
+        <f>B19*G19</f>
+        <v/>
+      </c>
+      <c r="J19" s="5" t="inlineStr">
+        <is>
           <t>Ontwerp in de map enclosure van het project; print in PETG of ASA (PLA wordt te zacht in de zon).</t>
         </is>
       </c>
     </row>
-    <row r="20">
-      <c r="A20" s="7" t="inlineStr">
+    <row r="21">
+      <c r="A21" s="7" t="inlineStr">
         <is>
           <t>Totaal verplicht</t>
         </is>
       </c>
-      <c r="H20" s="8">
-        <f>SUMIF(C5:C18,"Ja*",H5:H18)</f>
-        <v/>
-      </c>
-      <c r="I20" s="8">
-        <f>SUMIF(C5:C18,"Ja*",I5:I18)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
+      <c r="H21" s="8">
+        <f>SUMIF(C5:C19,"Ja*",H5:H19)</f>
+        <v/>
+      </c>
+      <c r="I21" s="8">
+        <f>SUMIF(C5:C19,"Ja*",I5:I19)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
         <is>
           <t>Totaal soms nodig en optioneel (sensoren tellen per stuk, zie opmerking)</t>
         </is>
       </c>
-      <c r="H21" s="9">
-        <f>SUM(H5:H18)-H20</f>
-        <v/>
-      </c>
-      <c r="I21" s="9">
-        <f>SUM(I5:I18)-I20</f>
+      <c r="H22" s="9">
+        <f>SUM(H5:H19)-H21</f>
+        <v/>
+      </c>
+      <c r="I22" s="9">
+        <f>SUM(I5:I19)-I21</f>
         <v/>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A4:J18"/>
+  <autoFilter ref="A4:J19"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Docs: same RTC cell advice everywhere
ML2032, ML2020 or ML1220 with a JST SH plug, like the Raspberry Pi 5 RTC
battery, with a polarity check before plugging in. Updated in README,
LEESMIJ, both compatibility lists, the quick start and the order list.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01DV9tygc5YXT9SuFFA2qLm4
</commit_message>
<xml_diff>
--- a/bestellijst.xlsx
+++ b/bestellijst.xlsx
@@ -596,7 +596,7 @@
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
         <is>
-          <t>Oplaadbare RTC-cel (ML1220) met stekkertje</t>
+          <t>Oplaadbare RTC-cel ML2032/ML2020 met JST-SH-stekker</t>
         </is>
       </c>
       <c r="B6" s="5" t="n">
@@ -614,14 +614,14 @@
       </c>
       <c r="E6" s="5" t="inlineStr">
         <is>
-          <t>Waveshare RTC battery ML1220</t>
+          <t>Raspberry Pi 5 RTC battery ML2032</t>
         </is>
       </c>
       <c r="F6" s="6" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="G6" s="6" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="H6" s="6">
         <f>B6*F6</f>
@@ -633,7 +633,7 @@
       </c>
       <c r="J6" s="5" t="inlineStr">
         <is>
-          <t>Sterk aangeraden: zonder cel is de tijd na elke stroomuitval weg. Als optie bij Waveshare mee te bestellen. Geen gewone CR2032: het board laadt de cel bij.</t>
+          <t>Sterk aangeraden: zonder cel is de tijd na elke stroomuitval weg. Zoals de RTC-batterij voor de Raspberry Pi 5. Controleer voor het insteken dat rood bij de + of 1 op het board uitkomt. Geen gewone CR2032.</t>
         </is>
       </c>
     </row>

</xml_diff>